<commit_message>
Update to local env data sets XLSX files
</commit_message>
<xml_diff>
--- a/datasets/local-data/FoE-local-env-data-LAD-2026.xlsx
+++ b/datasets/local-data/FoE-local-env-data-LAD-2026.xlsx
@@ -2791,7 +2791,7 @@
         <v>0.2957</v>
       </c>
       <c r="Q2" s="5" t="n">
-        <v>49</v>
+        <v>34</v>
       </c>
       <c r="R2" s="5" t="n">
         <v>419</v>
@@ -2962,7 +2962,7 @@
         <v>0.3313</v>
       </c>
       <c r="Q3" s="5" t="n">
-        <v>94</v>
+        <v>73</v>
       </c>
       <c r="R3" s="5" t="n">
         <v>671</v>
@@ -3133,7 +3133,7 @@
         <v>0.248</v>
       </c>
       <c r="Q4" s="5" t="n">
-        <v>84</v>
+        <v>72</v>
       </c>
       <c r="R4" s="5" t="n">
         <v>606</v>
@@ -3304,7 +3304,7 @@
         <v>0.2234</v>
       </c>
       <c r="Q5" s="5" t="n">
-        <v>155</v>
+        <v>132</v>
       </c>
       <c r="R5" s="5" t="n">
         <v>890</v>
@@ -3475,7 +3475,7 @@
         <v>0.2505</v>
       </c>
       <c r="Q6" s="5" t="n">
-        <v>113</v>
+        <v>95</v>
       </c>
       <c r="R6" s="5" t="n">
         <v>486</v>
@@ -3646,7 +3646,7 @@
         <v>0.2379</v>
       </c>
       <c r="Q7" s="5" t="n">
-        <v>66</v>
+        <v>57</v>
       </c>
       <c r="R7" s="5" t="n">
         <v>569</v>
@@ -3817,7 +3817,7 @@
         <v>0.1742</v>
       </c>
       <c r="Q8" s="5" t="n">
-        <v>235</v>
+        <v>163</v>
       </c>
       <c r="R8" s="5" t="n">
         <v>933</v>
@@ -3988,7 +3988,7 @@
         <v>0.2691</v>
       </c>
       <c r="Q9" s="5" t="n">
-        <v>67</v>
+        <v>59</v>
       </c>
       <c r="R9" s="5" t="n">
         <v>692</v>
@@ -4159,7 +4159,7 @@
         <v>0.3399</v>
       </c>
       <c r="Q10" s="5" t="n">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="R10" s="5" t="n">
         <v>627</v>
@@ -4330,7 +4330,7 @@
         <v>0.3505</v>
       </c>
       <c r="Q11" s="5" t="n">
-        <v>175</v>
+        <v>153</v>
       </c>
       <c r="R11" s="5" t="n">
         <v>1195</v>
@@ -4501,7 +4501,7 @@
         <v>0.1578</v>
       </c>
       <c r="Q12" s="5" t="n">
-        <v>251</v>
+        <v>223</v>
       </c>
       <c r="R12" s="5" t="n">
         <v>1539</v>
@@ -4672,7 +4672,7 @@
         <v>0.2692</v>
       </c>
       <c r="Q13" s="5" t="n">
-        <v>77</v>
+        <v>70</v>
       </c>
       <c r="R13" s="5" t="n">
         <v>696</v>
@@ -4843,7 +4843,7 @@
         <v>0.1845</v>
       </c>
       <c r="Q14" s="5" t="n">
-        <v>126</v>
+        <v>107</v>
       </c>
       <c r="R14" s="5" t="n">
         <v>747</v>
@@ -5014,7 +5014,7 @@
         <v>0.2395</v>
       </c>
       <c r="Q15" s="5" t="n">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="R15" s="5" t="n">
         <v>909</v>
@@ -5356,7 +5356,7 @@
         <v>0.3304</v>
       </c>
       <c r="Q17" s="5" t="n">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="R17" s="5" t="n">
         <v>1669</v>
@@ -5527,7 +5527,7 @@
         <v>0.1032</v>
       </c>
       <c r="Q18" s="5" t="n">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="R18" s="5" t="n">
         <v>179</v>
@@ -5698,7 +5698,7 @@
         <v>0.38</v>
       </c>
       <c r="Q19" s="5" t="n">
-        <v>318</v>
+        <v>302</v>
       </c>
       <c r="R19" s="5" t="n">
         <v>1447</v>
@@ -5869,7 +5869,7 @@
         <v>0.1444</v>
       </c>
       <c r="Q20" s="5" t="n">
-        <v>153</v>
+        <v>119</v>
       </c>
       <c r="R20" s="5" t="n">
         <v>834</v>
@@ -6040,7 +6040,7 @@
         <v>0.1872</v>
       </c>
       <c r="Q21" s="5" t="n">
-        <v>111</v>
+        <v>82</v>
       </c>
       <c r="R21" s="5" t="n">
         <v>843</v>
@@ -6211,7 +6211,7 @@
         <v>0.2732</v>
       </c>
       <c r="Q22" s="5" t="n">
-        <v>158</v>
+        <v>86</v>
       </c>
       <c r="R22" s="5" t="n">
         <v>1156</v>
@@ -6382,7 +6382,7 @@
         <v>0.1993</v>
       </c>
       <c r="Q23" s="5" t="n">
-        <v>121</v>
+        <v>103</v>
       </c>
       <c r="R23" s="5" t="n">
         <v>878</v>
@@ -6553,7 +6553,7 @@
         <v>0.2616</v>
       </c>
       <c r="Q24" s="5" t="n">
-        <v>187</v>
+        <v>193</v>
       </c>
       <c r="R24" s="5" t="n">
         <v>2123</v>
@@ -6724,7 +6724,7 @@
         <v>0.1496</v>
       </c>
       <c r="Q25" s="5" t="n">
-        <v>163</v>
+        <v>145</v>
       </c>
       <c r="R25" s="5" t="n">
         <v>972</v>
@@ -6895,7 +6895,7 @@
         <v>0.1235</v>
       </c>
       <c r="Q26" s="5" t="n">
-        <v>292</v>
+        <v>295</v>
       </c>
       <c r="R26" s="5" t="n">
         <v>1316</v>
@@ -7066,7 +7066,7 @@
         <v>0.2491</v>
       </c>
       <c r="Q27" s="5" t="n">
-        <v>365</v>
+        <v>291</v>
       </c>
       <c r="R27" s="5" t="n">
         <v>1181</v>
@@ -7237,7 +7237,7 @@
         <v>0.2323</v>
       </c>
       <c r="Q28" s="5" t="n">
-        <v>85</v>
+        <v>60</v>
       </c>
       <c r="R28" s="5" t="n">
         <v>613</v>
@@ -7579,7 +7579,7 @@
         <v>0.2265</v>
       </c>
       <c r="Q30" s="5" t="n">
-        <v>161</v>
+        <v>144</v>
       </c>
       <c r="R30" s="5" t="n">
         <v>965</v>
@@ -7750,7 +7750,7 @@
         <v>0.2498</v>
       </c>
       <c r="Q31" s="5" t="n">
-        <v>120</v>
+        <v>101</v>
       </c>
       <c r="R31" s="5" t="n">
         <v>1015</v>
@@ -8092,7 +8092,7 @@
         <v>0.1729</v>
       </c>
       <c r="Q33" s="5" t="n">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="R33" s="5" t="n">
         <v>783</v>
@@ -8263,7 +8263,7 @@
         <v>0.1924</v>
       </c>
       <c r="Q34" s="5" t="n">
-        <v>181</v>
+        <v>202</v>
       </c>
       <c r="R34" s="5" t="n">
         <v>1260</v>
@@ -8434,7 +8434,7 @@
         <v>0.1149</v>
       </c>
       <c r="Q35" s="5" t="n">
-        <v>125</v>
+        <v>144</v>
       </c>
       <c r="R35" s="5" t="n">
         <v>564</v>
@@ -8605,7 +8605,7 @@
         <v>0.1207</v>
       </c>
       <c r="Q36" s="5" t="n">
-        <v>326</v>
+        <v>298</v>
       </c>
       <c r="R36" s="5" t="n">
         <v>718</v>
@@ -8776,7 +8776,7 @@
         <v>0.2838</v>
       </c>
       <c r="Q37" s="5" t="n">
-        <v>317</v>
+        <v>320</v>
       </c>
       <c r="R37" s="5" t="n">
         <v>783</v>
@@ -8947,7 +8947,7 @@
         <v>0.2029</v>
       </c>
       <c r="Q38" s="5" t="n">
-        <v>118</v>
+        <v>89</v>
       </c>
       <c r="R38" s="5" t="n">
         <v>706</v>
@@ -9118,7 +9118,7 @@
         <v>0.127</v>
       </c>
       <c r="Q39" s="5" t="n">
-        <v>149</v>
+        <v>157</v>
       </c>
       <c r="R39" s="5" t="n">
         <v>682</v>
@@ -9289,7 +9289,7 @@
         <v>0.0902</v>
       </c>
       <c r="Q40" s="5" t="n">
-        <v>316</v>
+        <v>220</v>
       </c>
       <c r="R40" s="5" t="n">
         <v>808</v>
@@ -9460,7 +9460,7 @@
         <v>0.1711</v>
       </c>
       <c r="Q41" s="5" t="n">
-        <v>879</v>
+        <v>738</v>
       </c>
       <c r="R41" s="5" t="n">
         <v>1311</v>
@@ -9631,7 +9631,7 @@
         <v>0.3745</v>
       </c>
       <c r="Q42" s="5" t="n">
-        <v>575</v>
+        <v>526</v>
       </c>
       <c r="R42" s="5" t="n">
         <v>1229</v>
@@ -9802,7 +9802,7 @@
         <v>0.303</v>
       </c>
       <c r="Q43" s="5" t="n">
-        <v>255</v>
+        <v>151</v>
       </c>
       <c r="R43" s="5" t="n">
         <v>924</v>
@@ -9973,7 +9973,7 @@
         <v>0.2739</v>
       </c>
       <c r="Q44" s="5" t="n">
-        <v>126</v>
+        <v>97</v>
       </c>
       <c r="R44" s="5" t="n">
         <v>1126</v>
@@ -10144,7 +10144,7 @@
         <v>0.2076</v>
       </c>
       <c r="Q45" s="5" t="n">
-        <v>136</v>
+        <v>111</v>
       </c>
       <c r="R45" s="5" t="n">
         <v>619</v>
@@ -10315,7 +10315,7 @@
         <v>0.2413</v>
       </c>
       <c r="Q46" s="5" t="n">
-        <v>482</v>
+        <v>400</v>
       </c>
       <c r="R46" s="5" t="n">
         <v>2339</v>
@@ -10486,7 +10486,7 @@
         <v>0.1451</v>
       </c>
       <c r="Q47" s="5" t="n">
-        <v>327</v>
+        <v>240</v>
       </c>
       <c r="R47" s="5" t="n">
         <v>1813</v>
@@ -10657,7 +10657,7 @@
         <v>0.167</v>
       </c>
       <c r="Q48" s="5" t="n">
-        <v>281</v>
+        <v>237</v>
       </c>
       <c r="R48" s="5" t="n">
         <v>1604</v>
@@ -10828,7 +10828,7 @@
         <v>0.1381</v>
       </c>
       <c r="Q49" s="5" t="n">
-        <v>446</v>
+        <v>378</v>
       </c>
       <c r="R49" s="5" t="n">
         <v>1447</v>
@@ -10999,7 +10999,7 @@
         <v>0.1502</v>
       </c>
       <c r="Q50" s="5" t="n">
-        <v>883</v>
+        <v>752</v>
       </c>
       <c r="R50" s="5" t="n">
         <v>2542</v>
@@ -11170,7 +11170,7 @@
         <v>0.4176</v>
       </c>
       <c r="Q51" s="5" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="R51" s="5" t="n">
         <v>10</v>
@@ -11339,7 +11339,7 @@
         <v>0.1311</v>
       </c>
       <c r="Q52" s="5" t="n">
-        <v>491</v>
+        <v>440</v>
       </c>
       <c r="R52" s="5" t="n">
         <v>2276</v>
@@ -11510,7 +11510,7 @@
         <v>0.1819</v>
       </c>
       <c r="Q53" s="5" t="n">
-        <v>202</v>
+        <v>184</v>
       </c>
       <c r="R53" s="5" t="n">
         <v>834</v>
@@ -11681,7 +11681,7 @@
         <v>0.1127</v>
       </c>
       <c r="Q54" s="5" t="n">
-        <v>389</v>
+        <v>324</v>
       </c>
       <c r="R54" s="5" t="n">
         <v>1355</v>
@@ -11852,7 +11852,7 @@
         <v>0.1972</v>
       </c>
       <c r="Q55" s="5" t="n">
-        <v>611</v>
+        <v>557</v>
       </c>
       <c r="R55" s="5" t="n">
         <v>1437</v>
@@ -12023,7 +12023,7 @@
         <v>0.1938</v>
       </c>
       <c r="Q56" s="5" t="n">
-        <v>248</v>
+        <v>220</v>
       </c>
       <c r="R56" s="5" t="n">
         <v>1776</v>
@@ -12194,7 +12194,7 @@
         <v>0.1367</v>
       </c>
       <c r="Q57" s="5" t="n">
-        <v>447</v>
+        <v>313</v>
       </c>
       <c r="R57" s="5" t="n">
         <v>1691</v>
@@ -12365,7 +12365,7 @@
         <v>0.1148</v>
       </c>
       <c r="Q58" s="5" t="n">
-        <v>406</v>
+        <v>367</v>
       </c>
       <c r="R58" s="5" t="n">
         <v>2490</v>
@@ -12536,7 +12536,7 @@
         <v>0.1598</v>
       </c>
       <c r="Q59" s="5" t="n">
-        <v>305</v>
+        <v>267</v>
       </c>
       <c r="R59" s="5" t="n">
         <v>1617</v>
@@ -12707,7 +12707,7 @@
         <v>0.159</v>
       </c>
       <c r="Q60" s="5" t="n">
-        <v>375</v>
+        <v>347</v>
       </c>
       <c r="R60" s="5" t="n">
         <v>1909</v>
@@ -12878,7 +12878,7 @@
         <v>0.2032</v>
       </c>
       <c r="Q61" s="5" t="n">
-        <v>327</v>
+        <v>276</v>
       </c>
       <c r="R61" s="5" t="n">
         <v>1217</v>
@@ -13049,7 +13049,7 @@
         <v>0.1757</v>
       </c>
       <c r="Q62" s="5" t="n">
-        <v>579</v>
+        <v>476</v>
       </c>
       <c r="R62" s="5" t="n">
         <v>1003</v>
@@ -13220,7 +13220,7 @@
         <v>0.1571</v>
       </c>
       <c r="Q63" s="5" t="n">
-        <v>905</v>
+        <v>797</v>
       </c>
       <c r="R63" s="5" t="n">
         <v>2758</v>
@@ -13391,7 +13391,7 @@
         <v>0.1397</v>
       </c>
       <c r="Q64" s="5" t="n">
-        <v>533</v>
+        <v>471</v>
       </c>
       <c r="R64" s="5" t="n">
         <v>2554</v>
@@ -13562,7 +13562,7 @@
         <v>0.3437</v>
       </c>
       <c r="Q65" s="5" t="n">
-        <v>334</v>
+        <v>385</v>
       </c>
       <c r="R65" s="5" t="n">
         <v>659</v>
@@ -13733,7 +13733,7 @@
         <v>0.1203</v>
       </c>
       <c r="Q66" s="5" t="n">
-        <v>67</v>
+        <v>54</v>
       </c>
       <c r="R66" s="5" t="n">
         <v>402</v>
@@ -13904,7 +13904,7 @@
         <v>0.1594</v>
       </c>
       <c r="Q67" s="5" t="n">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="R67" s="5" t="n">
         <v>455</v>
@@ -14075,7 +14075,7 @@
         <v>0.1306</v>
       </c>
       <c r="Q68" s="5" t="n">
-        <v>176</v>
+        <v>121</v>
       </c>
       <c r="R68" s="5" t="n">
         <v>818</v>
@@ -14246,7 +14246,7 @@
         <v>0.1094</v>
       </c>
       <c r="Q69" s="5" t="n">
-        <v>254</v>
+        <v>175</v>
       </c>
       <c r="R69" s="5" t="n">
         <v>741</v>
@@ -14417,7 +14417,7 @@
         <v>0.1679</v>
       </c>
       <c r="Q70" s="5" t="n">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="R70" s="5" t="n">
         <v>561</v>
@@ -14588,7 +14588,7 @@
         <v>0.1851</v>
       </c>
       <c r="Q71" s="5" t="n">
-        <v>98</v>
+        <v>104</v>
       </c>
       <c r="R71" s="5" t="n">
         <v>364</v>
@@ -14759,7 +14759,7 @@
         <v>0.2392</v>
       </c>
       <c r="Q72" s="5" t="n">
-        <v>117</v>
+        <v>102</v>
       </c>
       <c r="R72" s="5" t="n">
         <v>461</v>
@@ -14930,7 +14930,7 @@
         <v>0.1303</v>
       </c>
       <c r="Q73" s="5" t="n">
-        <v>91</v>
+        <v>77</v>
       </c>
       <c r="R73" s="5" t="n">
         <v>314</v>
@@ -15101,7 +15101,7 @@
         <v>0.194</v>
       </c>
       <c r="Q74" s="5" t="n">
-        <v>57</v>
+        <v>47</v>
       </c>
       <c r="R74" s="5" t="n">
         <v>500</v>
@@ -15272,7 +15272,7 @@
         <v>0.1688</v>
       </c>
       <c r="Q75" s="5" t="n">
-        <v>71</v>
+        <v>58</v>
       </c>
       <c r="R75" s="5" t="n">
         <v>402</v>
@@ -15443,7 +15443,7 @@
         <v>0.1612</v>
       </c>
       <c r="Q76" s="5" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="R76" s="5" t="n">
         <v>462</v>
@@ -15614,7 +15614,7 @@
         <v>0.1112</v>
       </c>
       <c r="Q77" s="5" t="n">
-        <v>81</v>
+        <v>72</v>
       </c>
       <c r="R77" s="5" t="n">
         <v>501</v>
@@ -15785,7 +15785,7 @@
         <v>0.1357</v>
       </c>
       <c r="Q78" s="5" t="n">
-        <v>202</v>
+        <v>183</v>
       </c>
       <c r="R78" s="5" t="n">
         <v>686</v>
@@ -15956,7 +15956,7 @@
         <v>0.2539</v>
       </c>
       <c r="Q79" s="5" t="n">
-        <v>254</v>
+        <v>258</v>
       </c>
       <c r="R79" s="5" t="n">
         <v>602</v>
@@ -16127,7 +16127,7 @@
         <v>0.1306</v>
       </c>
       <c r="Q80" s="5" t="n">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="R80" s="5" t="n">
         <v>370</v>
@@ -16298,7 +16298,7 @@
         <v>0.1697</v>
       </c>
       <c r="Q81" s="5" t="n">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="R81" s="5" t="n">
         <v>442</v>
@@ -16469,7 +16469,7 @@
         <v>0.1171</v>
       </c>
       <c r="Q82" s="5" t="n">
-        <v>102</v>
+        <v>93</v>
       </c>
       <c r="R82" s="5" t="n">
         <v>399</v>
@@ -16640,7 +16640,7 @@
         <v>0.1442</v>
       </c>
       <c r="Q83" s="5" t="n">
-        <v>141</v>
+        <v>106</v>
       </c>
       <c r="R83" s="5" t="n">
         <v>602</v>
@@ -16811,7 +16811,7 @@
         <v>0.1373</v>
       </c>
       <c r="Q84" s="5" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="R84" s="5" t="n">
         <v>302</v>
@@ -16982,7 +16982,7 @@
         <v>0.1212</v>
       </c>
       <c r="Q85" s="5" t="n">
-        <v>76</v>
+        <v>50</v>
       </c>
       <c r="R85" s="5" t="n">
         <v>258</v>
@@ -17153,7 +17153,7 @@
         <v>0.2652</v>
       </c>
       <c r="Q86" s="5" t="n">
-        <v>76</v>
+        <v>63</v>
       </c>
       <c r="R86" s="5" t="n">
         <v>456</v>
@@ -17324,7 +17324,7 @@
         <v>0.2917</v>
       </c>
       <c r="Q87" s="5" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="R87" s="5" t="n">
         <v>399</v>
@@ -17495,7 +17495,7 @@
         <v>0.1879</v>
       </c>
       <c r="Q88" s="5" t="n">
-        <v>122</v>
+        <v>156</v>
       </c>
       <c r="R88" s="5" t="n">
         <v>445</v>
@@ -17666,7 +17666,7 @@
         <v>0.1601</v>
       </c>
       <c r="Q89" s="5" t="n">
-        <v>38</v>
+        <v>32</v>
       </c>
       <c r="R89" s="5" t="n">
         <v>417</v>
@@ -17837,7 +17837,7 @@
         <v>0.1058</v>
       </c>
       <c r="Q90" s="5" t="n">
-        <v>152</v>
+        <v>166</v>
       </c>
       <c r="R90" s="5" t="n">
         <v>724</v>
@@ -18008,7 +18008,7 @@
         <v>0.1873</v>
       </c>
       <c r="Q91" s="5" t="n">
-        <v>54</v>
+        <v>75</v>
       </c>
       <c r="R91" s="5" t="n">
         <v>837</v>
@@ -18179,7 +18179,7 @@
         <v>0.1374</v>
       </c>
       <c r="Q92" s="5" t="n">
-        <v>107</v>
+        <v>120</v>
       </c>
       <c r="R92" s="5" t="n">
         <v>703</v>
@@ -18350,7 +18350,7 @@
         <v>0.1374</v>
       </c>
       <c r="Q93" s="5" t="n">
-        <v>49</v>
+        <v>39</v>
       </c>
       <c r="R93" s="5" t="n">
         <v>343</v>
@@ -18521,7 +18521,7 @@
         <v>0.1496</v>
       </c>
       <c r="Q94" s="5" t="n">
-        <v>19</v>
+        <v>9</v>
       </c>
       <c r="R94" s="5" t="n">
         <v>395</v>
@@ -18692,7 +18692,7 @@
         <v>0.1487</v>
       </c>
       <c r="Q95" s="5" t="n">
-        <v>93</v>
+        <v>79</v>
       </c>
       <c r="R95" s="5" t="n">
         <v>814</v>
@@ -18863,7 +18863,7 @@
         <v>0.1824</v>
       </c>
       <c r="Q96" s="5" t="n">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="R96" s="5" t="n">
         <v>866</v>
@@ -19034,7 +19034,7 @@
         <v>0.1401</v>
       </c>
       <c r="Q97" s="5" t="n">
-        <v>100</v>
+        <v>79</v>
       </c>
       <c r="R97" s="5" t="n">
         <v>598</v>
@@ -19205,7 +19205,7 @@
         <v>0.2171</v>
       </c>
       <c r="Q98" s="5" t="n">
-        <v>39</v>
+        <v>49</v>
       </c>
       <c r="R98" s="5" t="n">
         <v>422</v>
@@ -19376,7 +19376,7 @@
         <v>0.1128</v>
       </c>
       <c r="Q99" s="5" t="n">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="R99" s="5" t="n">
         <v>300</v>
@@ -19547,7 +19547,7 @@
         <v>0.1296</v>
       </c>
       <c r="Q100" s="5" t="n">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="R100" s="5" t="n">
         <v>388</v>
@@ -19718,7 +19718,7 @@
         <v>0.2014</v>
       </c>
       <c r="Q101" s="5" t="n">
-        <v>80</v>
+        <v>50</v>
       </c>
       <c r="R101" s="5" t="n">
         <v>673</v>
@@ -19889,7 +19889,7 @@
         <v>0.0875</v>
       </c>
       <c r="Q102" s="5" t="n">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="R102" s="5" t="n">
         <v>411</v>
@@ -20060,7 +20060,7 @@
         <v>0.2008</v>
       </c>
       <c r="Q103" s="5" t="n">
-        <v>242</v>
+        <v>196</v>
       </c>
       <c r="R103" s="5" t="n">
         <v>528</v>
@@ -20231,7 +20231,7 @@
         <v>0.1099</v>
       </c>
       <c r="Q104" s="5" t="n">
-        <v>230</v>
+        <v>138</v>
       </c>
       <c r="R104" s="5" t="n">
         <v>402</v>
@@ -20402,7 +20402,7 @@
         <v>0.1218</v>
       </c>
       <c r="Q105" s="5" t="n">
-        <v>152</v>
+        <v>78</v>
       </c>
       <c r="R105" s="5" t="n">
         <v>392</v>
@@ -20573,7 +20573,7 @@
         <v>0.202</v>
       </c>
       <c r="Q106" s="5" t="n">
-        <v>125</v>
+        <v>103</v>
       </c>
       <c r="R106" s="5" t="n">
         <v>593</v>
@@ -20744,7 +20744,7 @@
         <v>0.1187</v>
       </c>
       <c r="Q107" s="5" t="n">
-        <v>239</v>
+        <v>297</v>
       </c>
       <c r="R107" s="5" t="n">
         <v>547</v>
@@ -20915,7 +20915,7 @@
         <v>0.1151</v>
       </c>
       <c r="Q108" s="5" t="n">
-        <v>96</v>
+        <v>46</v>
       </c>
       <c r="R108" s="5" t="n">
         <v>435</v>
@@ -21086,7 +21086,7 @@
         <v>0.1447</v>
       </c>
       <c r="Q109" s="5" t="n">
-        <v>166</v>
+        <v>148</v>
       </c>
       <c r="R109" s="5" t="n">
         <v>836</v>
@@ -21257,7 +21257,7 @@
         <v>0.0969</v>
       </c>
       <c r="Q110" s="5" t="n">
-        <v>61</v>
+        <v>49</v>
       </c>
       <c r="R110" s="5" t="n">
         <v>564</v>
@@ -21428,7 +21428,7 @@
         <v>0.1185</v>
       </c>
       <c r="Q111" s="5" t="n">
-        <v>127</v>
+        <v>114</v>
       </c>
       <c r="R111" s="5" t="n">
         <v>619</v>
@@ -21599,7 +21599,7 @@
         <v>0.1212</v>
       </c>
       <c r="Q112" s="5" t="n">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="R112" s="5" t="n">
         <v>502</v>
@@ -21770,7 +21770,7 @@
         <v>0.2065</v>
       </c>
       <c r="Q113" s="5" t="n">
-        <v>63</v>
+        <v>45</v>
       </c>
       <c r="R113" s="5" t="n">
         <v>362</v>
@@ -21941,7 +21941,7 @@
         <v>0.0785</v>
       </c>
       <c r="Q114" s="5" t="n">
-        <v>135</v>
+        <v>151</v>
       </c>
       <c r="R114" s="5" t="n">
         <v>446</v>
@@ -22112,7 +22112,7 @@
         <v>0.1806</v>
       </c>
       <c r="Q115" s="5" t="n">
-        <v>48</v>
+        <v>56</v>
       </c>
       <c r="R115" s="5" t="n">
         <v>552</v>
@@ -22283,7 +22283,7 @@
         <v>0.1165</v>
       </c>
       <c r="Q116" s="5" t="n">
-        <v>177</v>
+        <v>143</v>
       </c>
       <c r="R116" s="5" t="n">
         <v>771</v>
@@ -22454,7 +22454,7 @@
         <v>0.1634</v>
       </c>
       <c r="Q117" s="5" t="n">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="R117" s="5" t="n">
         <v>452</v>
@@ -22625,7 +22625,7 @@
         <v>0.1192</v>
       </c>
       <c r="Q118" s="5" t="n">
-        <v>101</v>
+        <v>110</v>
       </c>
       <c r="R118" s="5" t="n">
         <v>591</v>
@@ -22796,7 +22796,7 @@
         <v>0.1353</v>
       </c>
       <c r="Q119" s="5" t="n">
-        <v>219</v>
+        <v>179</v>
       </c>
       <c r="R119" s="5" t="n">
         <v>582</v>
@@ -22967,7 +22967,7 @@
         <v>0.1655</v>
       </c>
       <c r="Q120" s="5" t="n">
-        <v>88</v>
+        <v>62</v>
       </c>
       <c r="R120" s="5" t="n">
         <v>440</v>
@@ -23138,7 +23138,7 @@
         <v>0.145</v>
       </c>
       <c r="Q121" s="5" t="n">
-        <v>171</v>
+        <v>150</v>
       </c>
       <c r="R121" s="5" t="n">
         <v>694</v>
@@ -23309,7 +23309,7 @@
         <v>0.1551</v>
       </c>
       <c r="Q122" s="5" t="n">
-        <v>140</v>
+        <v>128</v>
       </c>
       <c r="R122" s="5" t="n">
         <v>479</v>
@@ -23480,7 +23480,7 @@
         <v>0.1548</v>
       </c>
       <c r="Q123" s="5" t="n">
-        <v>87</v>
+        <v>58</v>
       </c>
       <c r="R123" s="5" t="n">
         <v>596</v>
@@ -23651,7 +23651,7 @@
         <v>0.1248</v>
       </c>
       <c r="Q124" s="5" t="n">
-        <v>109</v>
+        <v>84</v>
       </c>
       <c r="R124" s="5" t="n">
         <v>416</v>
@@ -23822,7 +23822,7 @@
         <v>0.2242</v>
       </c>
       <c r="Q125" s="5" t="n">
-        <v>541</v>
+        <v>496</v>
       </c>
       <c r="R125" s="5" t="n">
         <v>458</v>
@@ -23993,7 +23993,7 @@
         <v>0.1438</v>
       </c>
       <c r="Q126" s="5" t="n">
-        <v>122</v>
+        <v>108</v>
       </c>
       <c r="R126" s="5" t="n">
         <v>608</v>
@@ -24164,7 +24164,7 @@
         <v>0.2083</v>
       </c>
       <c r="Q127" s="5" t="n">
-        <v>120</v>
+        <v>92</v>
       </c>
       <c r="R127" s="5" t="n">
         <v>703</v>
@@ -24335,7 +24335,7 @@
         <v>0.1685</v>
       </c>
       <c r="Q128" s="5" t="n">
-        <v>168</v>
+        <v>119</v>
       </c>
       <c r="R128" s="5" t="n">
         <v>530</v>
@@ -24506,7 +24506,7 @@
         <v>0.2007</v>
       </c>
       <c r="Q129" s="5" t="n">
-        <v>125</v>
+        <v>105</v>
       </c>
       <c r="R129" s="5" t="n">
         <v>521</v>
@@ -24677,7 +24677,7 @@
         <v>0.1966</v>
       </c>
       <c r="Q130" s="5" t="n">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="R130" s="5" t="n">
         <v>473</v>
@@ -24848,7 +24848,7 @@
         <v>0.1461</v>
       </c>
       <c r="Q131" s="5" t="n">
-        <v>101</v>
+        <v>89</v>
       </c>
       <c r="R131" s="5" t="n">
         <v>809</v>
@@ -25019,7 +25019,7 @@
         <v>0.1144</v>
       </c>
       <c r="Q132" s="5" t="n">
-        <v>98</v>
+        <v>83</v>
       </c>
       <c r="R132" s="5" t="n">
         <v>533</v>
@@ -25190,7 +25190,7 @@
         <v>0.2051</v>
       </c>
       <c r="Q133" s="5" t="n">
-        <v>189</v>
+        <v>159</v>
       </c>
       <c r="R133" s="5" t="n">
         <v>488</v>
@@ -25361,7 +25361,7 @@
         <v>0.1664</v>
       </c>
       <c r="Q134" s="5" t="n">
-        <v>121</v>
+        <v>95</v>
       </c>
       <c r="R134" s="5" t="n">
         <v>685</v>
@@ -25532,7 +25532,7 @@
         <v>0.2608</v>
       </c>
       <c r="Q135" s="5" t="n">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="R135" s="5" t="n">
         <v>617</v>
@@ -25703,7 +25703,7 @@
         <v>0.1231</v>
       </c>
       <c r="Q136" s="5" t="n">
-        <v>146</v>
+        <v>92</v>
       </c>
       <c r="R136" s="5" t="n">
         <v>594</v>
@@ -25874,7 +25874,7 @@
         <v>0.1552</v>
       </c>
       <c r="Q137" s="5" t="n">
-        <v>83</v>
+        <v>62</v>
       </c>
       <c r="R137" s="5" t="n">
         <v>514</v>
@@ -26045,7 +26045,7 @@
         <v>0.2926</v>
       </c>
       <c r="Q138" s="5" t="n">
-        <v>73</v>
+        <v>59</v>
       </c>
       <c r="R138" s="5" t="n">
         <v>424</v>
@@ -26216,7 +26216,7 @@
         <v>0.1464</v>
       </c>
       <c r="Q139" s="5" t="n">
-        <v>112</v>
+        <v>103</v>
       </c>
       <c r="R139" s="5" t="n">
         <v>525</v>
@@ -26387,7 +26387,7 @@
         <v>0.1679</v>
       </c>
       <c r="Q140" s="5" t="n">
-        <v>73</v>
+        <v>45</v>
       </c>
       <c r="R140" s="5" t="n">
         <v>368</v>
@@ -26558,7 +26558,7 @@
         <v>0.2534</v>
       </c>
       <c r="Q141" s="5" t="n">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="R141" s="5" t="n">
         <v>370</v>
@@ -26729,7 +26729,7 @@
         <v>0.2273</v>
       </c>
       <c r="Q142" s="5" t="n">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="R142" s="5" t="n">
         <v>640</v>
@@ -26900,7 +26900,7 @@
         <v>0.2327</v>
       </c>
       <c r="Q143" s="5" t="n">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="R143" s="5" t="n">
         <v>426</v>
@@ -27071,7 +27071,7 @@
         <v>0.2774</v>
       </c>
       <c r="Q144" s="5" t="n">
-        <v>83</v>
+        <v>74</v>
       </c>
       <c r="R144" s="5" t="n">
         <v>687</v>
@@ -27242,7 +27242,7 @@
         <v>0.1143</v>
       </c>
       <c r="Q145" s="5" t="n">
-        <v>61</v>
+        <v>55</v>
       </c>
       <c r="R145" s="5" t="n">
         <v>283</v>
@@ -27413,7 +27413,7 @@
         <v>0.1834</v>
       </c>
       <c r="Q146" s="5" t="n">
-        <v>92</v>
+        <v>78</v>
       </c>
       <c r="R146" s="5" t="n">
         <v>314</v>
@@ -27584,7 +27584,7 @@
         <v>0.1434</v>
       </c>
       <c r="Q147" s="5" t="n">
-        <v>120</v>
+        <v>106</v>
       </c>
       <c r="R147" s="5" t="n">
         <v>499</v>
@@ -27755,7 +27755,7 @@
         <v>0.1798</v>
       </c>
       <c r="Q148" s="5" t="n">
-        <v>104</v>
+        <v>119</v>
       </c>
       <c r="R148" s="5" t="n">
         <v>530</v>
@@ -27926,7 +27926,7 @@
         <v>0.1841</v>
       </c>
       <c r="Q149" s="5" t="n">
-        <v>107</v>
+        <v>100</v>
       </c>
       <c r="R149" s="5" t="n">
         <v>514</v>
@@ -28097,7 +28097,7 @@
         <v>0.1143</v>
       </c>
       <c r="Q150" s="5" t="n">
-        <v>119</v>
+        <v>102</v>
       </c>
       <c r="R150" s="5" t="n">
         <v>463</v>
@@ -28268,7 +28268,7 @@
         <v>0.1558</v>
       </c>
       <c r="Q151" s="5" t="n">
-        <v>134</v>
+        <v>108</v>
       </c>
       <c r="R151" s="5" t="n">
         <v>826</v>
@@ -28439,7 +28439,7 @@
         <v>0.0998</v>
       </c>
       <c r="Q152" s="5" t="n">
-        <v>102</v>
+        <v>95</v>
       </c>
       <c r="R152" s="5" t="n">
         <v>451</v>
@@ -28610,7 +28610,7 @@
         <v>0.1272</v>
       </c>
       <c r="Q153" s="5" t="n">
-        <v>73</v>
+        <v>84</v>
       </c>
       <c r="R153" s="5" t="n">
         <v>505</v>
@@ -28781,7 +28781,7 @@
         <v>0.1311</v>
       </c>
       <c r="Q154" s="5" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="R154" s="5" t="n">
         <v>234</v>
@@ -28952,7 +28952,7 @@
         <v>0.1261</v>
       </c>
       <c r="Q155" s="5" t="n">
-        <v>99</v>
+        <v>67</v>
       </c>
       <c r="R155" s="5" t="n">
         <v>485</v>
@@ -29123,7 +29123,7 @@
         <v>0.1679</v>
       </c>
       <c r="Q156" s="5" t="n">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="R156" s="5" t="n">
         <v>262</v>
@@ -29294,7 +29294,7 @@
         <v>0.195</v>
       </c>
       <c r="Q157" s="5" t="n">
-        <v>57</v>
+        <v>44</v>
       </c>
       <c r="R157" s="5" t="n">
         <v>314</v>
@@ -29465,7 +29465,7 @@
         <v>0.1669</v>
       </c>
       <c r="Q158" s="5" t="n">
-        <v>131</v>
+        <v>95</v>
       </c>
       <c r="R158" s="5" t="n">
         <v>639</v>
@@ -29636,7 +29636,7 @@
         <v>0.2838</v>
       </c>
       <c r="Q159" s="5" t="n">
-        <v>136</v>
+        <v>156</v>
       </c>
       <c r="R159" s="5" t="n">
         <v>454</v>
@@ -29807,7 +29807,7 @@
         <v>0.1142</v>
       </c>
       <c r="Q160" s="5" t="n">
-        <v>44</v>
+        <v>34</v>
       </c>
       <c r="R160" s="5" t="n">
         <v>533</v>
@@ -29978,7 +29978,7 @@
         <v>0.1289</v>
       </c>
       <c r="Q161" s="5" t="n">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="R161" s="5" t="n">
         <v>430</v>
@@ -30149,7 +30149,7 @@
         <v>0.146</v>
       </c>
       <c r="Q162" s="5" t="n">
-        <v>107</v>
+        <v>115</v>
       </c>
       <c r="R162" s="5" t="n">
         <v>641</v>
@@ -30320,7 +30320,7 @@
         <v>0.1413</v>
       </c>
       <c r="Q163" s="5" t="n">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="R163" s="5" t="n">
         <v>430</v>
@@ -30491,7 +30491,7 @@
         <v>0.1329</v>
       </c>
       <c r="Q164" s="5" t="n">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="R164" s="5" t="n">
         <v>638</v>
@@ -30662,7 +30662,7 @@
         <v>0.1098</v>
       </c>
       <c r="Q165" s="5" t="n">
-        <v>111</v>
+        <v>95</v>
       </c>
       <c r="R165" s="5" t="n">
         <v>596</v>
@@ -30833,7 +30833,7 @@
         <v>0.254</v>
       </c>
       <c r="Q166" s="5" t="n">
-        <v>101</v>
+        <v>83</v>
       </c>
       <c r="R166" s="5" t="n">
         <v>440</v>
@@ -31004,7 +31004,7 @@
         <v>0.1505</v>
       </c>
       <c r="Q167" s="5" t="n">
-        <v>149</v>
+        <v>125</v>
       </c>
       <c r="R167" s="5" t="n">
         <v>684</v>
@@ -31175,7 +31175,7 @@
         <v>0.146</v>
       </c>
       <c r="Q168" s="5" t="n">
-        <v>142</v>
+        <v>109</v>
       </c>
       <c r="R168" s="5" t="n">
         <v>454</v>
@@ -31346,7 +31346,7 @@
         <v>0.327</v>
       </c>
       <c r="Q169" s="5" t="n">
-        <v>187</v>
+        <v>136</v>
       </c>
       <c r="R169" s="5" t="n">
         <v>640</v>
@@ -31517,7 +31517,7 @@
         <v>0.1049</v>
       </c>
       <c r="Q170" s="5" t="n">
-        <v>164</v>
+        <v>121</v>
       </c>
       <c r="R170" s="5" t="n">
         <v>644</v>
@@ -31688,7 +31688,7 @@
         <v>0.206</v>
       </c>
       <c r="Q171" s="5" t="n">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="R171" s="5" t="n">
         <v>564</v>
@@ -31859,7 +31859,7 @@
         <v>0.1717</v>
       </c>
       <c r="Q172" s="5" t="n">
-        <v>138</v>
+        <v>118</v>
       </c>
       <c r="R172" s="5" t="n">
         <v>537</v>
@@ -32030,7 +32030,7 @@
         <v>0.1987</v>
       </c>
       <c r="Q173" s="5" t="n">
-        <v>80</v>
+        <v>64</v>
       </c>
       <c r="R173" s="5" t="n">
         <v>497</v>
@@ -32201,7 +32201,7 @@
         <v>0.1893</v>
       </c>
       <c r="Q174" s="5" t="n">
-        <v>66</v>
+        <v>92</v>
       </c>
       <c r="R174" s="5" t="n">
         <v>521</v>
@@ -32372,7 +32372,7 @@
         <v>0.2186</v>
       </c>
       <c r="Q175" s="5" t="n">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="R175" s="5" t="n">
         <v>493</v>
@@ -32543,7 +32543,7 @@
         <v>0.1616</v>
       </c>
       <c r="Q176" s="5" t="n">
-        <v>168</v>
+        <v>151</v>
       </c>
       <c r="R176" s="5" t="n">
         <v>554</v>
@@ -32714,7 +32714,7 @@
         <v>0.1345</v>
       </c>
       <c r="Q177" s="5" t="n">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="R177" s="5" t="n">
         <v>544</v>
@@ -32885,7 +32885,7 @@
         <v>0.1472</v>
       </c>
       <c r="Q178" s="5" t="n">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="R178" s="5" t="n">
         <v>731</v>
@@ -33056,7 +33056,7 @@
         <v>0.3211</v>
       </c>
       <c r="Q179" s="5" t="n">
-        <v>198</v>
+        <v>181</v>
       </c>
       <c r="R179" s="5" t="n">
         <v>726</v>
@@ -33227,7 +33227,7 @@
         <v>0.108</v>
       </c>
       <c r="Q180" s="5" t="n">
-        <v>117</v>
+        <v>97</v>
       </c>
       <c r="R180" s="5" t="n">
         <v>674</v>
@@ -33398,7 +33398,7 @@
         <v>0.1224</v>
       </c>
       <c r="Q181" s="5" t="n">
-        <v>197</v>
+        <v>177</v>
       </c>
       <c r="R181" s="5" t="n">
         <v>641</v>
@@ -33569,7 +33569,7 @@
         <v>0.115</v>
       </c>
       <c r="Q182" s="5" t="n">
-        <v>171</v>
+        <v>130</v>
       </c>
       <c r="R182" s="5" t="n">
         <v>524</v>
@@ -33740,7 +33740,7 @@
         <v>0.1692</v>
       </c>
       <c r="Q183" s="5" t="n">
-        <v>80</v>
+        <v>61</v>
       </c>
       <c r="R183" s="5" t="n">
         <v>452</v>
@@ -33911,7 +33911,7 @@
         <v>0.1849</v>
       </c>
       <c r="Q184" s="5" t="n">
-        <v>116</v>
+        <v>94</v>
       </c>
       <c r="R184" s="5" t="n">
         <v>561</v>
@@ -34082,7 +34082,7 @@
         <v>0.1264</v>
       </c>
       <c r="Q185" s="5" t="n">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="R185" s="5" t="n">
         <v>484</v>
@@ -34253,7 +34253,7 @@
         <v>0.1942</v>
       </c>
       <c r="Q186" s="5" t="n">
-        <v>143</v>
+        <v>116</v>
       </c>
       <c r="R186" s="5" t="n">
         <v>563</v>
@@ -34424,7 +34424,7 @@
         <v>0.1218</v>
       </c>
       <c r="Q187" s="5" t="n">
-        <v>96</v>
+        <v>85</v>
       </c>
       <c r="R187" s="5" t="n">
         <v>497</v>
@@ -34595,7 +34595,7 @@
         <v>0.1486</v>
       </c>
       <c r="Q188" s="5" t="n">
-        <v>112</v>
+        <v>122</v>
       </c>
       <c r="R188" s="5" t="n">
         <v>618</v>
@@ -34766,7 +34766,7 @@
         <v>0.1308</v>
       </c>
       <c r="Q189" s="5" t="n">
-        <v>55</v>
+        <v>37</v>
       </c>
       <c r="R189" s="5" t="n">
         <v>421</v>
@@ -34937,7 +34937,7 @@
         <v>0.1825</v>
       </c>
       <c r="Q190" s="5" t="n">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="R190" s="5" t="n">
         <v>353</v>
@@ -35108,7 +35108,7 @@
         <v>0.1165</v>
       </c>
       <c r="Q191" s="5" t="n">
-        <v>134</v>
+        <v>128</v>
       </c>
       <c r="R191" s="5" t="n">
         <v>421</v>
@@ -35279,7 +35279,7 @@
         <v>0.2481</v>
       </c>
       <c r="Q192" s="5" t="n">
-        <v>168</v>
+        <v>135</v>
       </c>
       <c r="R192" s="5" t="n">
         <v>613</v>
@@ -35450,7 +35450,7 @@
         <v>0.0977</v>
       </c>
       <c r="Q193" s="5" t="n">
-        <v>135</v>
+        <v>101</v>
       </c>
       <c r="R193" s="5" t="n">
         <v>475</v>
@@ -35621,7 +35621,7 @@
         <v>0.1114</v>
       </c>
       <c r="Q194" s="5" t="n">
-        <v>152</v>
+        <v>114</v>
       </c>
       <c r="R194" s="5" t="n">
         <v>617</v>
@@ -35792,7 +35792,7 @@
         <v>0.1426</v>
       </c>
       <c r="Q195" s="5" t="n">
-        <v>73</v>
+        <v>55</v>
       </c>
       <c r="R195" s="5" t="n">
         <v>360</v>
@@ -35963,7 +35963,7 @@
         <v>0.1383</v>
       </c>
       <c r="Q196" s="5" t="n">
-        <v>146</v>
+        <v>138</v>
       </c>
       <c r="R196" s="5" t="n">
         <v>656</v>
@@ -36134,7 +36134,7 @@
         <v>0.1154</v>
       </c>
       <c r="Q197" s="5" t="n">
-        <v>176</v>
+        <v>135</v>
       </c>
       <c r="R197" s="5" t="n">
         <v>388</v>
@@ -36305,7 +36305,7 @@
         <v>0.1346</v>
       </c>
       <c r="Q198" s="5" t="n">
-        <v>91</v>
+        <v>66</v>
       </c>
       <c r="R198" s="5" t="n">
         <v>685</v>
@@ -36476,7 +36476,7 @@
         <v>0.1388</v>
       </c>
       <c r="Q199" s="5" t="n">
-        <v>160</v>
+        <v>97</v>
       </c>
       <c r="R199" s="5" t="n">
         <v>397</v>
@@ -36647,7 +36647,7 @@
         <v>0.1473</v>
       </c>
       <c r="Q200" s="5" t="n">
-        <v>96</v>
+        <v>62</v>
       </c>
       <c r="R200" s="5" t="n">
         <v>457</v>
@@ -36989,7 +36989,7 @@
         <v>0.1127</v>
       </c>
       <c r="Q202" s="5" t="n">
-        <v>54</v>
+        <v>40</v>
       </c>
       <c r="R202" s="5" t="n">
         <v>393</v>
@@ -37160,7 +37160,7 @@
         <v>0.112</v>
       </c>
       <c r="Q203" s="5" t="n">
-        <v>115</v>
+        <v>107</v>
       </c>
       <c r="R203" s="5" t="n">
         <v>581</v>
@@ -37331,7 +37331,7 @@
         <v>0.1472</v>
       </c>
       <c r="Q204" s="5" t="n">
-        <v>172</v>
+        <v>196</v>
       </c>
       <c r="R204" s="5" t="n">
         <v>460</v>
@@ -37502,7 +37502,7 @@
         <v>0.1347</v>
       </c>
       <c r="Q205" s="5" t="n">
-        <v>112</v>
+        <v>81</v>
       </c>
       <c r="R205" s="5" t="n">
         <v>291</v>
@@ -37673,7 +37673,7 @@
         <v>0.1943</v>
       </c>
       <c r="Q206" s="5" t="n">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="R206" s="5" t="n">
         <v>606</v>
@@ -37844,7 +37844,7 @@
         <v>0.1459</v>
       </c>
       <c r="Q207" s="5" t="n">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="R207" s="5" t="n">
         <v>522</v>
@@ -38015,7 +38015,7 @@
         <v>0.1108</v>
       </c>
       <c r="Q208" s="5" t="n">
-        <v>196</v>
+        <v>182</v>
       </c>
       <c r="R208" s="5" t="n">
         <v>624</v>
@@ -38186,7 +38186,7 @@
         <v>0.166</v>
       </c>
       <c r="Q209" s="5" t="n">
-        <v>207</v>
+        <v>167</v>
       </c>
       <c r="R209" s="5" t="n">
         <v>673</v>
@@ -38357,7 +38357,7 @@
         <v>0.1847</v>
       </c>
       <c r="Q210" s="5" t="n">
-        <v>72</v>
+        <v>54</v>
       </c>
       <c r="R210" s="5" t="n">
         <v>284</v>
@@ -38528,7 +38528,7 @@
         <v>0.1686</v>
       </c>
       <c r="Q211" s="5" t="n">
-        <v>231</v>
+        <v>142</v>
       </c>
       <c r="R211" s="5" t="n">
         <v>738</v>
@@ -38699,7 +38699,7 @@
         <v>0.1408</v>
       </c>
       <c r="Q212" s="5" t="n">
-        <v>133</v>
+        <v>99</v>
       </c>
       <c r="R212" s="5" t="n">
         <v>563</v>
@@ -38870,7 +38870,7 @@
         <v>0.2059</v>
       </c>
       <c r="Q213" s="5" t="n">
-        <v>231</v>
+        <v>148</v>
       </c>
       <c r="R213" s="5" t="n">
         <v>530</v>
@@ -39041,7 +39041,7 @@
         <v>0.1124</v>
       </c>
       <c r="Q214" s="5" t="n">
-        <v>217</v>
+        <v>153</v>
       </c>
       <c r="R214" s="5" t="n">
         <v>657</v>
@@ -39212,7 +39212,7 @@
         <v>0.1237</v>
       </c>
       <c r="Q215" s="5" t="n">
-        <v>236</v>
+        <v>190</v>
       </c>
       <c r="R215" s="5" t="n">
         <v>694</v>
@@ -39383,7 +39383,7 @@
         <v>0.2184</v>
       </c>
       <c r="Q216" s="5" t="n">
-        <v>212</v>
+        <v>141</v>
       </c>
       <c r="R216" s="5" t="n">
         <v>493</v>
@@ -39554,7 +39554,7 @@
         <v>0.1137</v>
       </c>
       <c r="Q217" s="5" t="n">
-        <v>135</v>
+        <v>126</v>
       </c>
       <c r="R217" s="5" t="n">
         <v>442</v>
@@ -39725,7 +39725,7 @@
         <v>0.1185</v>
       </c>
       <c r="Q218" s="5" t="n">
-        <v>69</v>
+        <v>51</v>
       </c>
       <c r="R218" s="5" t="n">
         <v>360</v>
@@ -39896,7 +39896,7 @@
         <v>0.1762</v>
       </c>
       <c r="Q219" s="5" t="n">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="R219" s="5" t="n">
         <v>383</v>
@@ -40067,7 +40067,7 @@
         <v>0.2046</v>
       </c>
       <c r="Q220" s="5" t="n">
-        <v>166</v>
+        <v>159</v>
       </c>
       <c r="R220" s="5" t="n">
         <v>462</v>
@@ -40238,7 +40238,7 @@
         <v>0.1183</v>
       </c>
       <c r="Q221" s="5" t="n">
-        <v>139</v>
+        <v>135</v>
       </c>
       <c r="R221" s="5" t="n">
         <v>599</v>
@@ -40409,7 +40409,7 @@
         <v>0.1625</v>
       </c>
       <c r="Q222" s="5" t="n">
-        <v>48</v>
+        <v>40</v>
       </c>
       <c r="R222" s="5" t="n">
         <v>454</v>
@@ -40580,7 +40580,7 @@
         <v>0.1283</v>
       </c>
       <c r="Q223" s="5" t="n">
-        <v>88</v>
+        <v>73</v>
       </c>
       <c r="R223" s="5" t="n">
         <v>654</v>
@@ -40751,7 +40751,7 @@
         <v>0.1759</v>
       </c>
       <c r="Q224" s="5" t="n">
-        <v>310</v>
+        <v>221</v>
       </c>
       <c r="R224" s="5" t="n">
         <v>535</v>
@@ -40922,7 +40922,7 @@
         <v>0.1241</v>
       </c>
       <c r="Q225" s="5" t="n">
-        <v>150</v>
+        <v>117</v>
       </c>
       <c r="R225" s="5" t="n">
         <v>674</v>
@@ -41093,7 +41093,7 @@
         <v>0.2023</v>
       </c>
       <c r="Q226" s="5" t="n">
-        <v>106</v>
+        <v>125</v>
       </c>
       <c r="R226" s="5" t="n">
         <v>396</v>
@@ -41264,7 +41264,7 @@
         <v>0.1586</v>
       </c>
       <c r="Q227" s="5" t="n">
-        <v>211</v>
+        <v>186</v>
       </c>
       <c r="R227" s="5" t="n">
         <v>1086</v>
@@ -41606,7 +41606,7 @@
         <v>0.2477</v>
       </c>
       <c r="Q229" s="5" t="n">
-        <v>129</v>
+        <v>72</v>
       </c>
       <c r="R229" s="5" t="n">
         <v>1329</v>
@@ -41777,7 +41777,7 @@
         <v>0.2209</v>
       </c>
       <c r="Q230" s="5" t="n">
-        <v>70</v>
+        <v>55</v>
       </c>
       <c r="R230" s="5" t="n">
         <v>859</v>
@@ -41948,7 +41948,7 @@
         <v>0.3901</v>
       </c>
       <c r="Q231" s="5" t="n">
-        <v>549</v>
+        <v>424</v>
       </c>
       <c r="R231" s="5" t="n">
         <v>2549</v>
@@ -42119,7 +42119,7 @@
         <v>0.2764</v>
       </c>
       <c r="Q232" s="5" t="n">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="R232" s="5" t="n">
         <v>1082</v>
@@ -42290,7 +42290,7 @@
         <v>0.2626</v>
       </c>
       <c r="Q233" s="5" t="n">
-        <v>104</v>
+        <v>99</v>
       </c>
       <c r="R233" s="5" t="n">
         <v>1010</v>
@@ -42461,7 +42461,7 @@
         <v>0.3319</v>
       </c>
       <c r="Q234" s="5" t="n">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="R234" s="5" t="n">
         <v>1249</v>
@@ -42632,7 +42632,7 @@
         <v>0.1965</v>
       </c>
       <c r="Q235" s="5" t="n">
-        <v>196</v>
+        <v>138</v>
       </c>
       <c r="R235" s="5" t="n">
         <v>1316</v>
@@ -42803,7 +42803,7 @@
         <v>0.2609</v>
       </c>
       <c r="Q236" s="5" t="n">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="R236" s="5" t="n">
         <v>1031</v>
@@ -42974,7 +42974,7 @@
         <v>0.1927</v>
       </c>
       <c r="Q237" s="5" t="n">
-        <v>264</v>
+        <v>205</v>
       </c>
       <c r="R237" s="5" t="n">
         <v>1044</v>
@@ -43145,7 +43145,7 @@
         <v>0.2133</v>
       </c>
       <c r="Q238" s="5" t="n">
-        <v>193</v>
+        <v>153</v>
       </c>
       <c r="R238" s="5" t="n">
         <v>1491</v>
@@ -43316,7 +43316,7 @@
         <v>0.3121</v>
       </c>
       <c r="Q239" s="5" t="n">
-        <v>72</v>
+        <v>39</v>
       </c>
       <c r="R239" s="5" t="n">
         <v>700</v>
@@ -43487,7 +43487,7 @@
         <v>0.4007</v>
       </c>
       <c r="Q240" s="5" t="n">
-        <v>572</v>
+        <v>597</v>
       </c>
       <c r="R240" s="5" t="n">
         <v>2214</v>
@@ -43658,7 +43658,7 @@
         <v>0.2319</v>
       </c>
       <c r="Q241" s="5" t="n">
-        <v>89</v>
+        <v>48</v>
       </c>
       <c r="R241" s="5" t="n">
         <v>817</v>
@@ -43829,7 +43829,7 @@
         <v>0.2637</v>
       </c>
       <c r="Q242" s="5" t="n">
-        <v>112</v>
+        <v>78</v>
       </c>
       <c r="R242" s="5" t="n">
         <v>1243</v>
@@ -44000,7 +44000,7 @@
         <v>0.2507</v>
       </c>
       <c r="Q243" s="5" t="n">
-        <v>142</v>
+        <v>153</v>
       </c>
       <c r="R243" s="5" t="n">
         <v>1428</v>
@@ -44171,7 +44171,7 @@
         <v>0.2439</v>
       </c>
       <c r="Q244" s="5" t="n">
-        <v>210</v>
+        <v>169</v>
       </c>
       <c r="R244" s="5" t="n">
         <v>1381</v>
@@ -44342,7 +44342,7 @@
         <v>0.2299</v>
       </c>
       <c r="Q245" s="5" t="n">
-        <v>200</v>
+        <v>166</v>
       </c>
       <c r="R245" s="5" t="n">
         <v>1192</v>
@@ -44513,7 +44513,7 @@
         <v>0.3661</v>
       </c>
       <c r="Q246" s="5" t="n">
-        <v>277</v>
+        <v>283</v>
       </c>
       <c r="R246" s="5" t="n">
         <v>1371</v>
@@ -44684,7 +44684,7 @@
         <v>0.2781</v>
       </c>
       <c r="Q247" s="5" t="n">
-        <v>96</v>
+        <v>89</v>
       </c>
       <c r="R247" s="5" t="n">
         <v>931</v>
@@ -44855,7 +44855,7 @@
         <v>0.3276</v>
       </c>
       <c r="Q248" s="5" t="n">
-        <v>132</v>
+        <v>120</v>
       </c>
       <c r="R248" s="5" t="n">
         <v>656</v>
@@ -45026,7 +45026,7 @@
         <v>0.3092</v>
       </c>
       <c r="Q249" s="5" t="n">
-        <v>315</v>
+        <v>515</v>
       </c>
       <c r="R249" s="5" t="n">
         <v>1235</v>
@@ -45197,7 +45197,7 @@
         <v>0.3167</v>
       </c>
       <c r="Q250" s="5" t="n">
-        <v>1255</v>
+        <v>935</v>
       </c>
       <c r="R250" s="5" t="n">
         <v>5124</v>
@@ -45368,7 +45368,7 @@
         <v>0.2762</v>
       </c>
       <c r="Q251" s="5" t="n">
-        <v>2544</v>
+        <v>2272</v>
       </c>
       <c r="R251" s="5" t="n">
         <v>1585</v>
@@ -45539,7 +45539,7 @@
         <v>0.2049</v>
       </c>
       <c r="Q252" s="5" t="n">
-        <v>246</v>
+        <v>200</v>
       </c>
       <c r="R252" s="5" t="n">
         <v>1436</v>
@@ -45710,7 +45710,7 @@
         <v>0.2925</v>
       </c>
       <c r="Q253" s="5" t="n">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="R253" s="5" t="n">
         <v>1527</v>
@@ -45881,7 +45881,7 @@
         <v>0.1761</v>
       </c>
       <c r="Q254" s="5" t="n">
-        <v>434</v>
+        <v>354</v>
       </c>
       <c r="R254" s="5" t="n">
         <v>962</v>
@@ -46052,7 +46052,7 @@
         <v>0.2495</v>
       </c>
       <c r="Q255" s="5" t="n">
-        <v>103</v>
+        <v>84</v>
       </c>
       <c r="R255" s="5" t="n">
         <v>1269</v>
@@ -46223,7 +46223,7 @@
         <v>0.2849</v>
       </c>
       <c r="Q256" s="5" t="n">
-        <v>93</v>
+        <v>83</v>
       </c>
       <c r="R256" s="5" t="n">
         <v>1197</v>
@@ -46394,7 +46394,7 @@
         <v>0.2759</v>
       </c>
       <c r="Q257" s="5" t="n">
-        <v>313</v>
+        <v>240</v>
       </c>
       <c r="R257" s="5" t="n">
         <v>2462</v>
@@ -46565,7 +46565,7 @@
         <v>0.2451</v>
       </c>
       <c r="Q258" s="5" t="n">
-        <v>133</v>
+        <v>120</v>
       </c>
       <c r="R258" s="5" t="n">
         <v>917</v>
@@ -46736,7 +46736,7 @@
         <v>0.2267</v>
       </c>
       <c r="Q259" s="5" t="n">
-        <v>170</v>
+        <v>160</v>
       </c>
       <c r="R259" s="5" t="n">
         <v>1943</v>
@@ -46907,7 +46907,7 @@
         <v>0.2872</v>
       </c>
       <c r="Q260" s="5" t="n">
-        <v>679</v>
+        <v>620</v>
       </c>
       <c r="R260" s="5" t="n">
         <v>3645</v>
@@ -47078,7 +47078,7 @@
         <v>0.2282</v>
       </c>
       <c r="Q261" s="5" t="n">
-        <v>232</v>
+        <v>205</v>
       </c>
       <c r="R261" s="5" t="n">
         <v>1590</v>
@@ -47249,7 +47249,7 @@
         <v>0.324</v>
       </c>
       <c r="Q262" s="5" t="n">
-        <v>290</v>
+        <v>213</v>
       </c>
       <c r="R262" s="5" t="n">
         <v>875</v>
@@ -47420,7 +47420,7 @@
         <v>0.2275</v>
       </c>
       <c r="Q263" s="5" t="n">
-        <v>162</v>
+        <v>132</v>
       </c>
       <c r="R263" s="5" t="n">
         <v>1092</v>
@@ -47589,7 +47589,7 @@
         <v>0.2925</v>
       </c>
       <c r="Q264" s="5" t="n">
-        <v>403</v>
+        <v>315</v>
       </c>
       <c r="R264" s="5" t="n">
         <v>2519</v>
@@ -47758,7 +47758,7 @@
         <v>0.772</v>
       </c>
       <c r="Q265" s="5" t="n">
-        <v>95</v>
+        <v>84</v>
       </c>
       <c r="R265" s="5" t="n">
         <v>59</v>
@@ -47929,7 +47929,7 @@
         <v>0.3475</v>
       </c>
       <c r="Q266" s="5" t="n">
-        <v>165</v>
+        <v>118</v>
       </c>
       <c r="R266" s="5" t="n">
         <v>977</v>
@@ -48100,7 +48100,7 @@
         <v>0.2994</v>
       </c>
       <c r="Q267" s="5" t="n">
-        <v>1036</v>
+        <v>521</v>
       </c>
       <c r="R267" s="5" t="n">
         <v>1736</v>
@@ -48271,7 +48271,7 @@
         <v>0.2238</v>
       </c>
       <c r="Q268" s="5" t="n">
-        <v>220</v>
+        <v>206</v>
       </c>
       <c r="R268" s="5" t="n">
         <v>1102</v>
@@ -48442,7 +48442,7 @@
         <v>0.4409</v>
       </c>
       <c r="Q269" s="5" t="n">
-        <v>1157</v>
+        <v>1115</v>
       </c>
       <c r="R269" s="5" t="n">
         <v>1514</v>
@@ -48613,7 +48613,7 @@
         <v>0.2288</v>
       </c>
       <c r="Q270" s="5" t="n">
-        <v>200</v>
+        <v>220</v>
       </c>
       <c r="R270" s="5" t="n">
         <v>1455</v>
@@ -48784,7 +48784,7 @@
         <v>0.6365</v>
       </c>
       <c r="Q271" s="5" t="n">
-        <v>656</v>
+        <v>630</v>
       </c>
       <c r="R271" s="5" t="n">
         <v>971</v>
@@ -48955,7 +48955,7 @@
         <v>0.3362</v>
       </c>
       <c r="Q272" s="5" t="n">
-        <v>439</v>
+        <v>403</v>
       </c>
       <c r="R272" s="5" t="n">
         <v>1748</v>
@@ -49126,7 +49126,7 @@
         <v>0.368</v>
       </c>
       <c r="Q273" s="5" t="n">
-        <v>751</v>
+        <v>726</v>
       </c>
       <c r="R273" s="5" t="n">
         <v>1649</v>
@@ -49297,7 +49297,7 @@
         <v>0.3103</v>
       </c>
       <c r="Q274" s="5" t="n">
-        <v>289</v>
+        <v>234</v>
       </c>
       <c r="R274" s="5" t="n">
         <v>1439</v>
@@ -49468,7 +49468,7 @@
         <v>0.4313</v>
       </c>
       <c r="Q275" s="5" t="n">
-        <v>229</v>
+        <v>240</v>
       </c>
       <c r="R275" s="5" t="n">
         <v>1293</v>
@@ -49639,7 +49639,7 @@
         <v>0.6489</v>
       </c>
       <c r="Q276" s="5" t="n">
-        <v>1424</v>
+        <v>1084</v>
       </c>
       <c r="R276" s="5" t="n">
         <v>1157</v>
@@ -49810,7 +49810,7 @@
         <v>0.5746</v>
       </c>
       <c r="Q277" s="5" t="n">
-        <v>2662</v>
+        <v>2668</v>
       </c>
       <c r="R277" s="5" t="n">
         <v>818</v>
@@ -49981,7 +49981,7 @@
         <v>0.5273</v>
       </c>
       <c r="Q278" s="5" t="n">
-        <v>317</v>
+        <v>304</v>
       </c>
       <c r="R278" s="5" t="n">
         <v>1155</v>
@@ -50152,7 +50152,7 @@
         <v>0.2473</v>
       </c>
       <c r="Q279" s="5" t="n">
-        <v>73</v>
+        <v>85</v>
       </c>
       <c r="R279" s="5" t="n">
         <v>1158</v>
@@ -50323,7 +50323,7 @@
         <v>0.2153</v>
       </c>
       <c r="Q280" s="5" t="n">
-        <v>162</v>
+        <v>94</v>
       </c>
       <c r="R280" s="5" t="n">
         <v>1178</v>
@@ -50494,7 +50494,7 @@
         <v>0.223</v>
       </c>
       <c r="Q281" s="5" t="n">
-        <v>225</v>
+        <v>228</v>
       </c>
       <c r="R281" s="5" t="n">
         <v>1402</v>
@@ -50665,7 +50665,7 @@
         <v>0.3275</v>
       </c>
       <c r="Q282" s="5" t="n">
-        <v>608</v>
+        <v>611</v>
       </c>
       <c r="R282" s="5" t="n">
         <v>1300</v>
@@ -50836,7 +50836,7 @@
         <v>0.6688</v>
       </c>
       <c r="Q283" s="5" t="n">
-        <v>669</v>
+        <v>655</v>
       </c>
       <c r="R283" s="5" t="n">
         <v>969</v>
@@ -51007,7 +51007,7 @@
         <v>0.5831</v>
       </c>
       <c r="Q284" s="5" t="n">
-        <v>921</v>
+        <v>874</v>
       </c>
       <c r="R284" s="5" t="n">
         <v>648</v>
@@ -51178,7 +51178,7 @@
         <v>0.257</v>
       </c>
       <c r="Q285" s="5" t="n">
-        <v>397</v>
+        <v>409</v>
       </c>
       <c r="R285" s="5" t="n">
         <v>749</v>
@@ -51349,7 +51349,7 @@
         <v>0.5801</v>
       </c>
       <c r="Q286" s="5" t="n">
-        <v>668</v>
+        <v>617</v>
       </c>
       <c r="R286" s="5" t="n">
         <v>1387</v>
@@ -51520,7 +51520,7 @@
         <v>0.4769</v>
       </c>
       <c r="Q287" s="5" t="n">
-        <v>258</v>
+        <v>229</v>
       </c>
       <c r="R287" s="5" t="n">
         <v>1313</v>
@@ -51691,7 +51691,7 @@
         <v>0.3305</v>
       </c>
       <c r="Q288" s="5" t="n">
-        <v>869</v>
+        <v>809</v>
       </c>
       <c r="R288" s="5" t="n">
         <v>946</v>
@@ -51862,7 +51862,7 @@
         <v>0.5168</v>
       </c>
       <c r="Q289" s="5" t="n">
-        <v>359</v>
+        <v>258</v>
       </c>
       <c r="R289" s="5" t="n">
         <v>1593</v>
@@ -52033,7 +52033,7 @@
         <v>0.2751</v>
       </c>
       <c r="Q290" s="5" t="n">
-        <v>372</v>
+        <v>345</v>
       </c>
       <c r="R290" s="5" t="n">
         <v>1377</v>
@@ -52204,7 +52204,7 @@
         <v>0.2542</v>
       </c>
       <c r="Q291" s="5" t="n">
-        <v>1213</v>
+        <v>1002</v>
       </c>
       <c r="R291" s="5" t="n">
         <v>859</v>
@@ -52375,7 +52375,7 @@
         <v>0.6028</v>
       </c>
       <c r="Q292" s="5" t="n">
-        <v>1854</v>
+        <v>1869</v>
       </c>
       <c r="R292" s="5" t="n">
         <v>1387</v>
@@ -52546,7 +52546,7 @@
         <v>0.2281</v>
       </c>
       <c r="Q293" s="5" t="n">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="R293" s="5" t="n">
         <v>928</v>
@@ -52717,7 +52717,7 @@
         <v>0.6638</v>
       </c>
       <c r="Q294" s="5" t="n">
-        <v>2251</v>
+        <v>376</v>
       </c>
       <c r="R294" s="5" t="n">
         <v>1444</v>
@@ -52888,7 +52888,7 @@
         <v>0.4212</v>
       </c>
       <c r="Q295" s="5" t="n">
-        <v>1426</v>
+        <v>856</v>
       </c>
       <c r="R295" s="5" t="n">
         <v>1213</v>
@@ -53059,7 +53059,7 @@
         <v>0.4786</v>
       </c>
       <c r="Q296" s="5" t="n">
-        <v>1714</v>
+        <v>1473</v>
       </c>
       <c r="R296" s="5" t="n">
         <v>1457</v>
@@ -53230,7 +53230,7 @@
         <v>0.6622</v>
       </c>
       <c r="Q297" s="5" t="n">
-        <v>2783</v>
+        <v>2653</v>
       </c>
       <c r="R297" s="5" t="n">
         <v>929</v>
@@ -53395,7 +53395,7 @@
         <v>0.1498</v>
       </c>
       <c r="Q298" s="5" t="n">
-        <v>108</v>
+        <v>86</v>
       </c>
       <c r="R298" s="5" t="n">
         <v>305</v>
@@ -53542,7 +53542,7 @@
         <v>0.1766</v>
       </c>
       <c r="Q299" s="5" t="n">
-        <v>351</v>
+        <v>227</v>
       </c>
       <c r="R299" s="5" t="n">
         <v>524</v>
@@ -53689,7 +53689,7 @@
         <v>0.1852</v>
       </c>
       <c r="Q300" s="5" t="n">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="R300" s="5" t="n">
         <v>503</v>
@@ -53836,7 +53836,7 @@
         <v>0.188</v>
       </c>
       <c r="Q301" s="5" t="n">
-        <v>114</v>
+        <v>99</v>
       </c>
       <c r="R301" s="5" t="n">
         <v>427</v>
@@ -53983,7 +53983,7 @@
         <v>0.1457</v>
       </c>
       <c r="Q302" s="5" t="n">
-        <v>119</v>
+        <v>95</v>
       </c>
       <c r="R302" s="5" t="n">
         <v>685</v>
@@ -54130,7 +54130,7 @@
         <v>0.1905</v>
       </c>
       <c r="Q303" s="5" t="n">
-        <v>119</v>
+        <v>129</v>
       </c>
       <c r="R303" s="5" t="n">
         <v>598</v>
@@ -54277,7 +54277,7 @@
         <v>0.1573</v>
       </c>
       <c r="Q304" s="5" t="n">
-        <v>179</v>
+        <v>140</v>
       </c>
       <c r="R304" s="5" t="n">
         <v>321</v>
@@ -54424,7 +54424,7 @@
         <v>0.152</v>
       </c>
       <c r="Q305" s="5" t="n">
-        <v>276</v>
+        <v>248</v>
       </c>
       <c r="R305" s="5" t="n">
         <v>549</v>
@@ -54571,7 +54571,7 @@
         <v>0.154</v>
       </c>
       <c r="Q306" s="5" t="n">
-        <v>255</v>
+        <v>199</v>
       </c>
       <c r="R306" s="5" t="n">
         <v>835</v>
@@ -54718,7 +54718,7 @@
         <v>0.2264</v>
       </c>
       <c r="Q307" s="5" t="n">
-        <v>247</v>
+        <v>201</v>
       </c>
       <c r="R307" s="5" t="n">
         <v>1084</v>
@@ -54865,7 +54865,7 @@
         <v>0.2094</v>
       </c>
       <c r="Q308" s="5" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="R308" s="5" t="n">
         <v>628</v>
@@ -55012,7 +55012,7 @@
         <v>0.1823</v>
       </c>
       <c r="Q309" s="5" t="n">
-        <v>166</v>
+        <v>136</v>
       </c>
       <c r="R309" s="5" t="n">
         <v>645</v>
@@ -55159,7 +55159,7 @@
         <v>0.1659</v>
       </c>
       <c r="Q310" s="5" t="n">
-        <v>179</v>
+        <v>217</v>
       </c>
       <c r="R310" s="5" t="n">
         <v>592</v>
@@ -55306,7 +55306,7 @@
         <v>0.2599</v>
       </c>
       <c r="Q311" s="5" t="n">
-        <v>251</v>
+        <v>213</v>
       </c>
       <c r="R311" s="5" t="n">
         <v>1685</v>
@@ -55453,7 +55453,7 @@
         <v>0.2222</v>
       </c>
       <c r="Q312" s="5" t="n">
-        <v>239</v>
+        <v>204</v>
       </c>
       <c r="R312" s="5" t="n">
         <v>1060</v>
@@ -55600,7 +55600,7 @@
         <v>0.2033</v>
       </c>
       <c r="Q313" s="5" t="n">
-        <v>110</v>
+        <v>73</v>
       </c>
       <c r="R313" s="5" t="n">
         <v>775</v>
@@ -55747,7 +55747,7 @@
         <v>0.2297</v>
       </c>
       <c r="Q314" s="5" t="n">
-        <v>92</v>
+        <v>78</v>
       </c>
       <c r="R314" s="5" t="n">
         <v>296</v>
@@ -55894,7 +55894,7 @@
         <v>0.1963</v>
       </c>
       <c r="Q315" s="5" t="n">
-        <v>105</v>
+        <v>90</v>
       </c>
       <c r="R315" s="5" t="n">
         <v>411</v>
@@ -56041,7 +56041,7 @@
         <v>0.1294</v>
       </c>
       <c r="Q316" s="5" t="n">
-        <v>171</v>
+        <v>134</v>
       </c>
       <c r="R316" s="5" t="n">
         <v>416</v>
@@ -56188,7 +56188,7 @@
         <v>0.2259</v>
       </c>
       <c r="Q317" s="5" t="n">
-        <v>291</v>
+        <v>186</v>
       </c>
       <c r="R317" s="5" t="n">
         <v>719</v>
@@ -56335,7 +56335,7 @@
         <v>0.131</v>
       </c>
       <c r="Q318" s="5" t="n">
-        <v>205</v>
+        <v>151</v>
       </c>
       <c r="R318" s="5" t="n">
         <v>591</v>
@@ -56482,7 +56482,7 @@
         <v>0.2504</v>
       </c>
       <c r="Q319" s="7" t="n">
-        <v>58</v>
+        <v>40</v>
       </c>
       <c r="R319" s="7" t="n">
         <v>257</v>

</xml_diff>